<commit_message>
Add preorders workflow and packaging docs
</commit_message>
<xml_diff>
--- a/plantilla_productos_cardbastion.xlsx
+++ b/plantilla_productos_cardbastion.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:X3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,7 +422,55 @@
         <v>stock</v>
       </c>
       <c r="H1" t="str">
+        <v>min_stock</v>
+      </c>
+      <c r="I1" t="str">
         <v>image</v>
+      </c>
+      <c r="J1" t="str">
+        <v>product_type</v>
+      </c>
+      <c r="K1" t="str">
+        <v>game</v>
+      </c>
+      <c r="L1" t="str">
+        <v>card_name</v>
+      </c>
+      <c r="M1" t="str">
+        <v>set_name</v>
+      </c>
+      <c r="N1" t="str">
+        <v>set_code</v>
+      </c>
+      <c r="O1" t="str">
+        <v>collector_number</v>
+      </c>
+      <c r="P1" t="str">
+        <v>finish</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>language</v>
+      </c>
+      <c r="R1" t="str">
+        <v>card_condition</v>
+      </c>
+      <c r="S1" t="str">
+        <v>starcity_url</v>
+      </c>
+      <c r="T1" t="str">
+        <v>starcity_variant_key</v>
+      </c>
+      <c r="U1" t="str">
+        <v>starcity_price_usd</v>
+      </c>
+      <c r="V1" t="str">
+        <v>pricing_mode</v>
+      </c>
+      <c r="W1" t="str">
+        <v>pricing_formula_type</v>
+      </c>
+      <c r="X1" t="str">
+        <v>pricing_formula_value</v>
       </c>
     </row>
     <row r="2">
@@ -433,10 +481,10 @@
         <v>750200001</v>
       </c>
       <c r="C2" t="str">
-        <v>Booster Pokémon Temporal Forces</v>
+        <v>Booster Pokemon Temporal Forces</v>
       </c>
       <c r="D2" t="str">
-        <v>Pokémon</v>
+        <v>Pokemon</v>
       </c>
       <c r="E2">
         <v>129</v>
@@ -447,39 +495,135 @@
       <c r="G2">
         <v>24</v>
       </c>
-      <c r="H2" t="str">
-        <v/>
+      <c r="H2">
+        <v>4</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v>normal</v>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2" t="str">
+        <v>manual</v>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>MTG-210</v>
+        <v>MTG-SINGLE-001</v>
       </c>
       <c r="B3" t="str">
-        <v>750200002</v>
+        <v/>
       </c>
       <c r="C3" t="str">
-        <v>Play Booster Final Fantasy</v>
+        <v>Lightning Bolt</v>
       </c>
       <c r="D3" t="str">
-        <v>Magic</v>
+        <v>Singles</v>
       </c>
       <c r="E3">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="F3">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="G3">
-        <v>18</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v>single</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Magic: The Gathering</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Lightning Bolt</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Magic 2010</v>
+      </c>
+      <c r="N3" t="str">
+        <v>M10</v>
+      </c>
+      <c r="O3" t="str">
+        <v>146</v>
+      </c>
+      <c r="P3" t="str">
+        <v>nonfoil</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>EN</v>
+      </c>
+      <c r="R3" t="str">
+        <v>NM</v>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3" t="str">
+        <v>starcity_formula</v>
+      </c>
+      <c r="W3" t="str">
+        <v>multiplier</v>
+      </c>
+      <c r="X3">
+        <v>1.15</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>